<commit_message>
Update data package at: 2026-09-28T13:24:29Z
</commit_message>
<xml_diff>
--- a/data/checks-planejamento.xlsx
+++ b/data/checks-planejamento.xlsx
@@ -352,7 +352,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B108"/>
+  <dimension ref="A1:B93"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1471,231 +1471,6 @@
       <c r="B93" t="inlineStr">
         <is>
           <t>A uo 5261 está com setor divergente na base ações-planejamento (INFRAESTRTURA, MOBILIDADE E PARCERIAS) em relação à tabela auxiliar setor-governo da loa (INFRAESTRUTURA, MOBILIDADE E PARCERIAS).</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>check_valores_sigplan_programas</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>A uo 2311, 
-programa 7, 
-área temática 03AT03 está com valor 
-de meta orçamentária do ano 0, base programas (R$ 216.248.265,00) diferente da base ações-planejamento (R$ 151.136.947,00). Diferença de R$ -65111318.</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>check_valores_sigplan_programas</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>A uo 1191, 
-programa 20, 
-área temática 01AT01 está com valor 
-de meta orçamentária do ano 0, base programas (R$ 13.239.000,00) diferente da base ações-planejamento (R$ 13.238.000,00). Diferença de R$ -1000.</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>check_valores_sigplan_programas</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>A uo 1371, 
-programa 21, 
-área temática 11AT11 está com valor 
-de meta orçamentária do ano 0, base programas (R$ 3.418.369.851,00) diferente da base ações-planejamento (R$ 115.369.851,00). Diferença de R$ -3.303e+09.</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>check_valores_sigplan_programas</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>A uo 2151, 
-programa 42, 
-área temática 03AT03 está com valor 
-de meta orçamentária do ano 0, base programas (R$ 31.775.244,00) diferente da base ações-planejamento (R$ 31.765.244,00). Diferença de R$ -10000.</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>check_valores_sigplan_programas</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>A uo 4291, 
-programa 60, 
-área temática 04AT04 está com valor 
-de meta orçamentária do ano 0, base programas (R$ 702.771.556,00) diferente da base ações-planejamento (R$ 702.247.087,00). Diferença de R$ -524469.</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>check_valores_sigplan_programas</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>A uo 1481, 
-programa 68, 
-área temática 10AT10 está com valor 
-de meta orçamentária do ano 0, base programas (R$ 40.387.963,00) diferente da base ações-planejamento (R$ 27.201.811,00). Diferença de R$ -13186152.</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>check_valores_sigplan_programas</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>A uo 1481, 
-programa 83, 
-área temática 10AT10 está com valor 
-de meta orçamentária do ano 0, base programas (R$ 1.562.570,00) diferente da base ações-planejamento (R$ 1.233.792,00). Diferença de R$ -328778.</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>check_valores_sigplan_programas</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>A uo 1301, 
-programa 99, 
-área temática 05AT05 está com valor 
-de meta orçamentária do ano 0, base programas (R$ 37.444.335,00) diferente da base ações-planejamento (R$ 36.529.088,00). Diferença de R$ -915247.</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>check_valores_sigplan_programas</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>A uo 1491, 
-programa 119, 
-área temática 12AT12 está com valor 
-de meta orçamentária do ano 0, base programas (R$ 35.963.734,00) diferente da base ações-planejamento (R$ 35.962.734,00). Diferença de R$ -1000.</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>check_valores_sigplan_programas</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>A uo 1221, 
-programa 133, 
-área temática 02AT02 está com valor 
-de meta orçamentária do ano 0, base programas (R$ 498.121.008,00) diferente da base ações-planejamento (R$ 495.758.569,00). Diferença de R$ -2362439.</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>check_valores_sigplan_programas</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>A uo 1251, 
-programa 136, 
-área temática 03AT03 está com valor 
-de meta orçamentária do ano 0, base programas (R$ 257.268.346,00) diferente da base ações-planejamento (R$ 257.267.346,00). Diferença de R$ -1000.</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>check_valores_sigplan_programas</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>A uo 1071, 
-programa 139, 
-área temática 12AT12 está com valor 
-de meta orçamentária do ano 0, base programas (R$ 207.973.317,00) diferente da base ações-planejamento (R$ 207.973.316,00). Diferença de R$ -1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>check_valores_sigplan_programas</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>A uo 2481, 
-programa 161, 
-área temática 08AT08 está com valor 
-de meta orçamentária do ano 0, base programas (R$ 406.412.088,00) diferente da base ações-planejamento (R$ 406.411.088,00). Diferença de R$ -1000.</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>check_valores_sigplan_programas</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>A uo 1261, 
-programa 165, 
-área temática 03AT03 está com valor 
-de meta orçamentária do ano 0, base programas (R$ 44.615.293,00) diferente da base ações-planejamento (R$ 43.575.293,00). Diferença de R$ -1040000.</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>check_valores_sigplan_programas</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>A uo 1501, 
-programa 705, 
-área temática 08AT08 está com valor 
-de meta orçamentária do ano 0, base programas (R$ 72.198.856.106,00) diferente da base ações-planejamento (R$ 72.198.854.106,00). Diferença de R$ -2000.</t>
         </is>
       </c>
     </row>
@@ -1706,7 +1481,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1861,16 +1636,6 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>check_valores_sigplan_programas</t>
-        </is>
-      </c>
-      <c r="B16">
-        <v>15</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update data package at: 2026-09-29T15:29:54Z
</commit_message>
<xml_diff>
--- a/data/checks-planejamento.xlsx
+++ b/data/checks-planejamento.xlsx
@@ -352,7 +352,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B93"/>
+  <dimension ref="A1:B86"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -666,7 +666,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>A Fonte de Recurso 60 está com os valores totais de receita e despesa diferentes nas bases. R$ 4.506.993.690,00 na base orçamento fiscal da receita, e 5.326.603.517,00 na qdd fiscal. A diferença é de R$ -819609827.</t>
+          <t>A Fonte de Recurso 60 está com os valores totais de receita e despesa diferentes nas bases. R$ 4.506.993.690,00 na base orçamento fiscal da receita, e 3.692.974.668,00 na qdd fiscal. A diferença é de R$ 814019022.</t>
         </is>
       </c>
     </row>
@@ -1213,84 +1213,84 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>check_repasse_recursos</t>
+          <t>check_setor_governo</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>A uo 1251, fonte 60, grupo 3, ipu 2 está com valor de despesa na base qdd-fiscal (R$ 263.715.306,00) diferente do valor repassado para essa mesma uo  na base repasse-recursos (R$  NA). Diferença de R$  NA.</t>
+          <t>A uo 1301 está com setor divergente na base ações-planejamento (INFRAESTRTURA, MOBILIDADE E PARCERIAS) em relação à tabela auxiliar setor-governo da loa (INFRAESTRUTURA, MOBILIDADE E PARCERIAS).</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>check_repasse_recursos</t>
+          <t>check_setor_governo</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>A uo 1251, fonte 60, grupo 4, ipu 2 está com valor de despesa na base qdd-fiscal (R$ 5.358.422,00) diferente do valor repassado para essa mesma uo  na base repasse-recursos (R$  NA). Diferença de R$  NA.</t>
+          <t>A uo 1917 está com setor divergente na base ações-planejamento (NA) em relação à tabela auxiliar setor-governo da loa (FAZENDA).</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>check_repasse_recursos</t>
+          <t>check_setor_governo</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>A uo 1451, fonte 60, grupo 3, ipu 2 está com valor de despesa na base qdd-fiscal (R$ 1.072.922.038,00) diferente do valor repassado para essa mesma uo  na base repasse-recursos (R$  NA). Diferença de R$  NA.</t>
+          <t>A uo 2301 está com setor divergente na base ações-planejamento (INFRAESTRTURA, MOBILIDADE E PARCERIAS) em relação à tabela auxiliar setor-governo da loa (INFRAESTRUTURA, MOBILIDADE E PARCERIAS).</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>check_repasse_recursos</t>
+          <t>check_setor_governo</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>A uo 1451, fonte 60, grupo 3, ipu 2 está com valor de despesa na base qdd-fiscal (R$ 46.826.403,00) diferente do valor repassado para essa mesma uo  na base repasse-recursos (R$  NA). Diferença de R$  NA.</t>
+          <t>A uo 2431 está com setor divergente na base ações-planejamento (INFRAESTRTURA, MOBILIDADE E PARCERIAS) em relação à tabela auxiliar setor-governo da loa (INFRAESTRUTURA, MOBILIDADE E PARCERIAS).</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>check_repasse_recursos</t>
+          <t>check_setor_governo</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>A uo 1451, fonte 60, grupo 4, ipu 2 está com valor de despesa na base qdd-fiscal (R$ 910.719,00) diferente do valor repassado para essa mesma uo  na base repasse-recursos (R$  NA). Diferença de R$  NA.</t>
+          <t>A uo 2461 está com setor divergente na base ações-planejamento (INFRAESTRTURA, MOBILIDADE E PARCERIAS) em relação à tabela auxiliar setor-governo da loa (INFRAESTRUTURA, MOBILIDADE E PARCERIAS).</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>check_repasse_recursos</t>
+          <t>check_setor_governo</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>A uo 1511, fonte 60, grupo 3, ipu 2 está com valor de despesa na base qdd-fiscal (R$ 217.067.440,00) diferente do valor repassado para essa mesma uo  na base repasse-recursos (R$  NA). Diferença de R$  NA.</t>
+          <t>A uo 2471 está com setor divergente na base ações-planejamento (INFRAESTRTURA, MOBILIDADE E PARCERIAS) em relação à tabela auxiliar setor-governo da loa (INFRAESTRUTURA, MOBILIDADE E PARCERIAS).</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>check_repasse_recursos</t>
+          <t>check_setor_governo</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>A uo 1511, fonte 60, grupo 4, ipu 2 está com valor de despesa na base qdd-fiscal (R$ 26.828.521,00) diferente do valor repassado para essa mesma uo  na base repasse-recursos (R$  NA). Diferença de R$  NA.</t>
+          <t>A uo 2481 está com setor divergente na base ações-planejamento (PLANEJAMENTO E GESTÃO) em relação à tabela auxiliar setor-governo da loa (NA).</t>
         </is>
       </c>
     </row>
@@ -1302,7 +1302,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>A uo 1301 está com setor divergente na base ações-planejamento (INFRAESTRTURA, MOBILIDADE E PARCERIAS) em relação à tabela auxiliar setor-governo da loa (INFRAESTRUTURA, MOBILIDADE E PARCERIAS).</t>
+          <t>A uo 2781 está com setor divergente na base ações-planejamento (NA) em relação à tabela auxiliar setor-governo da loa (PLANEJAMENTO E GESTÃO).</t>
         </is>
       </c>
     </row>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>A uo 1917 está com setor divergente na base ações-planejamento (NA) em relação à tabela auxiliar setor-governo da loa (FAZENDA).</t>
+          <t>A uo 4171 está com setor divergente na base ações-planejamento (NA) em relação à tabela auxiliar setor-governo da loa (AGRICULTURA, PECUÁRIA E ABASTECIMENTO).</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>A uo 2301 está com setor divergente na base ações-planejamento (INFRAESTRTURA, MOBILIDADE E PARCERIAS) em relação à tabela auxiliar setor-governo da loa (INFRAESTRUTURA, MOBILIDADE E PARCERIAS).</t>
+          <t>A uo 4331 está com setor divergente na base ações-planejamento (INFRAESTRTURA, MOBILIDADE E PARCERIAS) em relação à tabela auxiliar setor-governo da loa (INFRAESTRUTURA, MOBILIDADE E PARCERIAS).</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>A uo 2431 está com setor divergente na base ações-planejamento (INFRAESTRTURA, MOBILIDADE E PARCERIAS) em relação à tabela auxiliar setor-governo da loa (INFRAESTRUTURA, MOBILIDADE E PARCERIAS).</t>
+          <t>A uo 4381 está com setor divergente na base ações-planejamento (INFRAESTRTURA, MOBILIDADE E PARCERIAS) em relação à tabela auxiliar setor-governo da loa (INFRAESTRUTURA, MOBILIDADE E PARCERIAS).</t>
         </is>
       </c>
     </row>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>A uo 2461 está com setor divergente na base ações-planejamento (INFRAESTRTURA, MOBILIDADE E PARCERIAS) em relação à tabela auxiliar setor-governo da loa (INFRAESTRUTURA, MOBILIDADE E PARCERIAS).</t>
+          <t>A uo 4531 está com setor divergente na base ações-planejamento (NA) em relação à tabela auxiliar setor-governo da loa (DESENVOLVIMENTO ECONÔMICO).</t>
         </is>
       </c>
     </row>
@@ -1362,7 +1362,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>A uo 2471 está com setor divergente na base ações-planejamento (INFRAESTRTURA, MOBILIDADE E PARCERIAS) em relação à tabela auxiliar setor-governo da loa (INFRAESTRUTURA, MOBILIDADE E PARCERIAS).</t>
+          <t>A uo 4631 está com setor divergente na base ações-planejamento (INFRAESTRTURA, MOBILIDADE E PARCERIAS) em relação à tabela auxiliar setor-governo da loa (INFRAESTRUTURA, MOBILIDADE E PARCERIAS).</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>A uo 2481 está com setor divergente na base ações-planejamento (PLANEJAMENTO E GESTÃO) em relação à tabela auxiliar setor-governo da loa (NA).</t>
+          <t>A uo 4641 está com setor divergente na base ações-planejamento (INFRAESTRTURA, MOBILIDADE E PARCERIAS) em relação à tabela auxiliar setor-governo da loa (INFRAESTRUTURA, MOBILIDADE E PARCERIAS).</t>
         </is>
       </c>
     </row>
@@ -1385,90 +1385,6 @@
         </is>
       </c>
       <c r="B86" t="inlineStr">
-        <is>
-          <t>A uo 2781 está com setor divergente na base ações-planejamento (NA) em relação à tabela auxiliar setor-governo da loa (PLANEJAMENTO E GESTÃO).</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>check_setor_governo</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>A uo 4171 está com setor divergente na base ações-planejamento (NA) em relação à tabela auxiliar setor-governo da loa (AGRICULTURA, PECUÁRIA E ABASTECIMENTO).</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>check_setor_governo</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>A uo 4331 está com setor divergente na base ações-planejamento (INFRAESTRTURA, MOBILIDADE E PARCERIAS) em relação à tabela auxiliar setor-governo da loa (INFRAESTRUTURA, MOBILIDADE E PARCERIAS).</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>check_setor_governo</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>A uo 4381 está com setor divergente na base ações-planejamento (INFRAESTRTURA, MOBILIDADE E PARCERIAS) em relação à tabela auxiliar setor-governo da loa (INFRAESTRUTURA, MOBILIDADE E PARCERIAS).</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>check_setor_governo</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>A uo 4531 está com setor divergente na base ações-planejamento (NA) em relação à tabela auxiliar setor-governo da loa (DESENVOLVIMENTO ECONÔMICO).</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>check_setor_governo</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>A uo 4631 está com setor divergente na base ações-planejamento (INFRAESTRTURA, MOBILIDADE E PARCERIAS) em relação à tabela auxiliar setor-governo da loa (INFRAESTRUTURA, MOBILIDADE E PARCERIAS).</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>check_setor_governo</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>A uo 4641 está com setor divergente na base ações-planejamento (INFRAESTRTURA, MOBILIDADE E PARCERIAS) em relação à tabela auxiliar setor-governo da loa (INFRAESTRUTURA, MOBILIDADE E PARCERIAS).</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>check_setor_governo</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
         <is>
           <t>A uo 5261 está com setor divergente na base ações-planejamento (INFRAESTRTURA, MOBILIDADE E PARCERIAS) em relação à tabela auxiliar setor-governo da loa (INFRAESTRUTURA, MOBILIDADE E PARCERIAS).</t>
         </is>
@@ -1481,7 +1397,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1619,20 +1535,10 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>check_repasse_recursos</t>
+          <t>check_setor_governo</t>
         </is>
       </c>
       <c r="B14">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>check_setor_governo</t>
-        </is>
-      </c>
-      <c r="B15">
         <v>15</v>
       </c>
     </row>

</xml_diff>